<commit_message>
Algo tresholds tests results
</commit_message>
<xml_diff>
--- a/tresholds.xlsx
+++ b/tresholds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c64c0255ed6b9c45/Desktop/Diagnosis_System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="11_AD4DADEC636C813AC809E4C38859613C5ADEDD89" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5CC60D8-5F72-405A-BD00-A1B48A7D4432}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="11_AD4DADEC636C813AC809E4C38859613C5ADEDD89" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E95338E5-D749-41DF-9FE2-1DB3ED44E0D8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>MSO 0</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>0.0001</t>
+  </si>
+  <si>
+    <t>najlepsze wyniki</t>
   </si>
 </sst>
 </file>
@@ -588,32 +591,32 @@
         <v>6.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E19" s="2">
         <v>5.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E23">
         <v>6.9999999999999994E-5</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>14</v>
       </c>
@@ -626,8 +629,12 @@
       <c r="E26" t="s">
         <v>17</v>
       </c>
+      <c r="G26" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>